<commit_message>
Add News sheet and end_date/next_position to People; add emit_news
</commit_message>
<xml_diff>
--- a/site_data.xlsx
+++ b/site_data.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publications" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collaborators" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funders" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Publications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="People" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Collaborators" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Funders" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="News" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5115,7 +5116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5139,7 +5140,8 @@
     <col width="36" customWidth="1" min="19" max="19"/>
     <col width="32" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="6" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="36" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -5250,6 +5252,16 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>next_position</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>show</t>
         </is>
       </c>
@@ -5360,7 +5372,17 @@
           <t>e.g. 2021-2024 (alumni only)</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD (alumni only)</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>Position upon leaving (alumni only)</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>yes/no</t>
         </is>
@@ -5462,7 +5484,7 @@
           <t>https://ilas.shisu.edu.cn/21/0f/c18209a205071/page.htm</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6217,4 +6239,330 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>featured</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tag_zh</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tag_en</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>title_zh</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>title_en</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>summary_zh</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>summary_en</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>body_zh</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>body_en</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>show</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or YYYY-MM</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>yes / blank (highlight on home sidebar)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Chinese tag (e.g. 国际合作招募)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>English tag</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Chinese title</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>English title</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Chinese summary (shown on home sidebar)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>English summary</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Chinese body (full text on News page)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>English body</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>External link (optional)</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>yes/no</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>国际合作招募</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Int'l Recruitment</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>上海市国际合作研究项目 2026 年度招募外籍青年学者</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026 Shanghai Sci-tech Co-research Program: call for foreign young scientists</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>面向 45 岁以下外籍青年学者，单项资助 40 万人民币，资助期 2 年。课题组优先合作方向：言语情绪、神经语用、跨语言认知。</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Open to foreign scientists under 45. Each project funded at RMB 400,000 over 2 years. Priority areas: vocal emotion, neuropragmatics, cross-linguistic cognition.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>由上海市科学技术委员会（STCSM）发布，面向全球 45 岁以下、在海外高校或研究机构任职的青年学者。项目期内需在上海累计驻留不少于 6 个月（含一次连续 3 个月）。申请期：2026 年 1 月 28 日 9:00 — 2026 年 12 月 31 日 16:30（北京时间）。课题组提供合作方案打磨、签证及行政支持。意向合作请直接邮件联系蒋晓鸣教授。</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Released by the Shanghai Science and Technology Commission (STCSM). Eligible to foreign scientists under 45 holding a position at an overseas university or research institute. Requires a cumulative 6-month stay in Shanghai (with one continuous 3-month block) during the project. Application window: 9:00 28 Jan 2026 — 16:30 31 Dec 2026 (Beijing time). The lab provides proposal-shaping, visa and administrative support — write directly to Prof. Jiang to discuss.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://xiaomingjiang.wordpress.com/</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>博士招生</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ph.D. Admissions</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>中国研究 (CSP) 博士奖学金：持续招收国际博士生</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>China Studies Program (CSP) Ph.D. Fellowship: ongoing intake</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>面向国际申请者的全额博士奖学金，研究方向涵盖心理语言学、神经语言学、跨文化交际等。</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Fully-funded Ph.D. scholarship for international applicants in psycholinguistics, neurolinguistics, and intercultural communication.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>申请人须具备相关学科本科或硕士背景，提交研究计划与推荐信。课题组每年接收 1–2 名 CSP 博士生。具体申请流程请参考上外研究生院相关页面，意向请提前邮件联系。</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Applicants should hold a relevant Bachelor's/Master's degree and submit a research proposal with letters of recommendation. The lab accepts 1–2 CSP fellows per year. See SISU Graduate School pages for the formal process; please email in advance to express interest.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://xiaomingjiang.wordpress.com/looking-for-a-phd-through-2022-2023-china-studies-program-csp-ph-d-fellowship/</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>学术活动</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Conference</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>中国心理语言学年会 (China Psycholinguistics Annual Conference)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>China Psycholinguistics Annual Conference</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>上外语言科学研究院定期承办的国内顶级心理语言学学术会议。</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>The leading domestic psycholinguistics meeting, regularly hosted by SISU ILAS.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>课题组成员积极参与会议组织与报告，欢迎合作者联系交流。</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Lab members are actively involved in organization and presentations; collaborators are welcome to get in touch.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly ORCID + xlsx sync
</commit_message>
<xml_diff>
--- a/site_data.xlsx
+++ b/site_data.xlsx
@@ -688,16 +688,22 @@
           <t>https://doi.org/10.1016/j.lingua.2026.104185</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -715,6 +721,7 @@
           <t>Tianze Xu; Xiaoming Jiang; Volker Dellwo</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>preprint</t>
@@ -730,16 +737,22 @@
           <t>https://doi.org/10.31234/osf.io/4zrwy_v3</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -777,16 +790,22 @@
           <t>https://doi.org/10.1016/j.neuroimage.2026.121987</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -824,16 +843,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2026.109493</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -871,16 +896,22 @@
           <t>https://doi.org/10.1044/2025_JSLHR-25-00294</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -898,6 +929,7 @@
           <t>Wenjun Chen; Marc D. Pell; Xiaoming Jiang</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>preprint</t>
@@ -913,16 +945,22 @@
           <t>https://doi.org/10.64898/2026.04.08.716483</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -960,16 +998,22 @@
           <t>https://doi.org/10.1016/j.bandl.2026.105723</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1007,16 +1051,22 @@
           <t>https://doi.org/10.1016/j.chbah.2026.100261</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1054,16 +1104,22 @@
           <t>https://doi.org/10.1371/journal.pone.0327529</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1101,16 +1157,22 @@
           <t>https://doi.org/10.1038/s41597-025-06110-5</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1148,16 +1210,22 @@
           <t>https://doi.org/10.1044/2025_JSLHR-24-00849</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1195,16 +1263,22 @@
           <t>https://doi.org/10.1186/s40359-025-03522-1</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1222,6 +1296,7 @@
           <t>Wenjun Chen; Marc D. Pell; Xiaoming Jiang</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>preprint</t>
@@ -1237,16 +1312,22 @@
           <t>https://doi.org/10.20944/preprints202510.1492.v1</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1284,16 +1365,22 @@
           <t>https://doi.org/10.1016/j.neuroimage.2025.121253</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1331,16 +1418,22 @@
           <t>https://doi.org/10.3390/languages10060119</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1378,16 +1471,22 @@
           <t>https://doi.org/10.3758/s13428-025-02608-3</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1425,16 +1524,22 @@
           <t>https://doi.org/10.1121/10.0032400</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1472,16 +1577,22 @@
           <t>https://doi.org/10.1016/j.tics.2024.08.005</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1519,16 +1630,22 @@
           <t>https://doi.org/10.3390/bs14080686</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1566,16 +1683,22 @@
           <t>https://doi.org/10.1057/s41599-024-03502-7</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1613,16 +1736,22 @@
           <t>https://doi.org/10.3390/brainsci14030264</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1660,16 +1789,22 @@
           <t>https://doi.org/10.1044/2024_JSLHR-23-00553</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1707,16 +1842,22 @@
           <t>https://doi.org/10.3791/66913</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1754,16 +1895,22 @@
           <t>https://doi.org/10.1016/j.aip.2024.102167</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1781,6 +1928,7 @@
           <t>Wenjun Chen; Xiaoming Jiang</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>preprint</t>
@@ -1796,16 +1944,22 @@
           <t>https://doi.org/10.20944/preprints202312.0807.v1</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1843,6 +1997,9 @@
           <t>https://doi.org/10.20944/preprints202303.0517.v1</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>yes</t>
@@ -1853,11 +2010,13 @@
           <t>journal</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1895,16 +2054,22 @@
           <t>https://doi.org/10.1007/s12144-022-03528-7</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1942,16 +2107,22 @@
           <t>https://doi.org/10.1007/s10919-023-00428-7</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1989,16 +2160,22 @@
           <t>https://doi.org/10.3389/fpsyg.2023.1289045</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2036,16 +2213,22 @@
           <t>https://doi.org/10.1016/j.actpsy.2023.103955</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2083,16 +2266,22 @@
           <t>https://doi.org/10.3390/brainsci13121724</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2130,16 +2319,22 @@
           <t>https://doi.org/10.1038/s41597-022-01811-7</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2177,16 +2372,22 @@
           <t>https://doi.org/10.1016/j.jneuroling.2023.101143</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2224,16 +2425,22 @@
           <t>https://doi.org/10.1016/j.pragma.2023.07.005</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2271,16 +2478,22 @@
           <t>https://doi.org/10.1073/pnas.2111091119</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2318,16 +2531,22 @@
           <t>https://doi.org/10.21437/Interspeech.2022-10531</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2365,16 +2584,22 @@
           <t>https://doi.org/10.1016/j.cortex.2021.12.017</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2412,16 +2637,22 @@
           <t>https://doi.org/10.1073/pnas.2213828119</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2449,16 +2680,24 @@
           <t>journal-article</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2496,16 +2735,22 @@
           <t>https://doi.org/10.1109/ISCSLP57327.2022.10037951</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2543,16 +2788,22 @@
           <t>https://doi.org/10.1007/s42761-022-00128-3</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2590,16 +2841,22 @@
           <t>https://doi.org/10.1016/j.pscychresns.2022.111489</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2637,16 +2894,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2022.108254</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2684,16 +2947,22 @@
           <t>https://doi.org/10.3389/fnins.2022.953315</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2731,16 +3000,22 @@
           <t>https://doi.org/10.3389/fpsyg.2022.1028106</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2778,16 +3053,22 @@
           <t>https://doi.org/10.1080/17470919.2021.1938667</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2825,16 +3106,22 @@
           <t>https://doi.org/10.3758/s13415-020-00849-7</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2872,16 +3159,22 @@
           <t>https://doi.org/10.1177/0022022121990897</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2894,6 +3187,7 @@
           <t>An alternative structure rescues failed semantics? Strong global expectancy reduces local-mismatch N400 in Chinese flexible structures</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>Neuropsychologia</t>
@@ -2914,16 +3208,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2020.107380</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2961,16 +3261,22 @@
           <t>https://doi.org/10.1080/23273798.2020.1781213</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3008,16 +3314,22 @@
           <t>https://doi.org/10.1016/j.brainres.2020.146855</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3055,16 +3367,22 @@
           <t>https://doi.org/10.1016/j.biopsycho.2020.107909</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3102,16 +3420,22 @@
           <t>https://doi.org/10.1177/1747021819865833</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3124,6 +3448,7 @@
           <t>Eye Movements Reveal Delayed Use of Construction-Based Pragmatic Information During Online Sentence Reading: A Case of Chinese Lian…dou Construction</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>Frontiers in Psychology</t>
@@ -3144,16 +3469,22 @@
           <t>https://doi.org/10.3389/fpsyg.2019.02211</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3166,6 +3497,7 @@
           <t>Commentary: A Neural Mechanism of Social Categorization</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Frontiers in Neuroscience</t>
@@ -3186,16 +3518,22 @@
           <t>https://doi.org/10.3389/fnins.2019.00368</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3208,6 +3546,7 @@
           <t>Single-trial Based EEG Classification of the Dynamic Representation of Speaker Stance: A Preliminary Study with Representational Similarity Analysis</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>NeuroManagement and Intelligent Computing Method on Multimodal Interaction on - ICMI '19</t>
@@ -3228,16 +3567,22 @@
           <t>https://doi.org/10.1145/3357160.3357672</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3275,6 +3620,9 @@
           <t>https://doi.org/10.31234/osf.io/8dr23</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3285,11 +3633,13 @@
           <t>journal</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3327,16 +3677,22 @@
           <t>https://doi.org/10.1016/j.specom.2018.06.004</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3374,16 +3730,22 @@
           <t>https://doi.org/10.1016/j.neuroimage.2018.07.042</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3421,16 +3783,22 @@
           <t>https://doi.org/10.21437/SpeechProsody.2018-55</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3468,16 +3836,22 @@
           <t>https://doi.org/10.1002/hbm.23630</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3515,16 +3889,22 @@
           <t>https://doi.org/10.1016/j.snb.2017.01.052</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3562,16 +3942,22 @@
           <t>https://doi.org/10.1016/j.bandl.2017.04.005</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3609,16 +3995,22 @@
           <t>https://doi.org/10.1002/hbm.23633</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3656,16 +4048,22 @@
           <t>https://doi.org/10.1016/j.specom.2017.01.011</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3703,16 +4101,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2015.12.008</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3750,16 +4154,22 @@
           <t>https://doi.org/10.1037/xhp0000240</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3797,16 +4207,22 @@
           <t>https://doi.org/10.1037/xhp0000043</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3844,16 +4260,22 @@
           <t>https://doi.org/10.1016/j.cortex.2015.02.002</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3891,16 +4313,22 @@
           <t>https://doi.org/10.1080/23273798.2015.1005636</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3938,16 +4366,22 @@
           <t>https://doi.org/10.3389/fnhum.2014.00873</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3985,16 +4419,22 @@
           <t>https://doi.org/10.1093/scan/nst091</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4022,16 +4462,24 @@
           <t>conference-paper</t>
         </is>
       </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4069,16 +4517,22 @@
           <t>https://doi.org/10.1016/j.brainres.2012.10.042</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4116,16 +4570,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2013.06.009</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4163,16 +4623,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2013.07.021</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4210,16 +4676,22 @@
           <t>https://doi.org/10.1016/j.bandc.2012.11.002</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4257,16 +4729,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2012.04.016</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4304,16 +4782,22 @@
           <t>https://doi.org/10.1016/j.neuroscience.2011.10.035</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4351,16 +4835,22 @@
           <t>https://doi.org/10.1016/j.brainres.2011.06.061</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4398,16 +4888,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2010.02.001</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4445,16 +4941,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2009.01.013</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4492,16 +4994,22 @@
           <t>https://doi.org/10.1016/j.neuropsychologia.2009.02.020</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr">
         <is>
           <t>0000-0002-5171-9774</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4868,8 +5376,6 @@
           <t>Professor · Doctoral Supervisor</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>主要从事心理与神经语言学的科学研究与人才培养工作。研究方向：心理与神经语言学、实验语言学、言语交际与言语障碍、嗓音编码与解码、神经语用学。</t>

</xml_diff>